<commit_message>
Fix ZBX UI Update
</commit_message>
<xml_diff>
--- a/traffic_capt.xlsx
+++ b/traffic_capt.xlsx
@@ -25,36 +25,7 @@
     <t>AM16224607741106N</t>
   </si>
   <si>
-    <t xml:space="preserve">Error saat proses site AM16224607741106N: Login gagal: Message: element click intercepted: Element &lt;button type="submit" class="mt-1 v-btn v-btn--block v-btn--disabled v-btn--has-bg theme--light v-size--default" disabled="disabled"&gt;...&lt;/button&gt; is not clickable at point (769, 518). Other element would receive the click: &lt;div class="py-3"&gt;...&lt;/div&gt;
-  (Session info: chrome=132.0.6834.83)
-Stacktrace:
-	GetHandleVerifier [0x008B74A3+25091]
-	(No symbol) [0x0083DC04]
-	(No symbol) [0x0071B373]
-	(No symbol) [0x007654B8]
-	(No symbol) [0x007638C4]
-	(No symbol) [0x00761467]
-	(No symbol) [0x0076076A]
-	(No symbol) [0x007553A5]
-	(No symbol) [0x00781F0C]
-	(No symbol) [0x00754E44]
-	(No symbol) [0x007821A4]
-	(No symbol) [0x0079B49E]
-	(No symbol) [0x00781CA6]
-	(No symbol) [0x007531D5]
-	(No symbol) [0x0075435D]
-	GetHandleVerifier [0x00BB07C3+3142947]
-	GetHandleVerifier [0x00BC1A2B+3213195]
-	GetHandleVerifier [0x00BBC412+3191154]
-	GetHandleVerifier [0x00958720+685184]
-	(No symbol) [0x00846E1D]
-	(No symbol) [0x00843E18]
-	(No symbol) [0x00843FB6]
-	(No symbol) [0x008366F0]
-	BaseThreadInitThunk [0x767C5D49+25]
-	RtlInitializeExceptionChain [0x7796CDEB+107]
-	RtlGetAppContainerNamedObjectPath [0x7796CD71+561]
-</t>
+    <t>Done Capture</t>
   </si>
 </sst>
 </file>

</xml_diff>